<commit_message>
create null_threshold parameter for fine tuning filtering of data before loading
</commit_message>
<xml_diff>
--- a/column_list_by_processing_method.xlsx
+++ b/column_list_by_processing_method.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JLopez.SOLIDIATECH\de_projects\noaa_eda\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40001_{1943ED91-69B0-4B42-B736-C7B212CA377F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080826D9-3FE2-48D3-8D2E-AAFDA5E564D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1275" yWindow="-120" windowWidth="27645" windowHeight="16440"/>
+    <workbookView xWindow="1275" yWindow="-120" windowWidth="27645" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="360">
   <si>
     <t>'column0'</t>
   </si>
@@ -1086,13 +1087,43 @@
   </si>
   <si>
     <t>TURTLE</t>
+  </si>
+  <si>
+    <t>before</t>
+  </si>
+  <si>
+    <t>after</t>
+  </si>
+  <si>
+    <t>(5654239, 49)</t>
+  </si>
+  <si>
+    <t>(7143914, 35)</t>
+  </si>
+  <si>
+    <t>(3638646, 110)</t>
+  </si>
+  <si>
+    <t>(5654239, 28)</t>
+  </si>
+  <si>
+    <t>(5654239, 27)</t>
+  </si>
+  <si>
+    <t>(7143914, 19)</t>
+  </si>
+  <si>
+    <t>(3638646, 42)</t>
+  </si>
+  <si>
+    <t>(7143914, 21)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1106,8 +1137,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC1C4CE"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1123,6 +1160,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1148,7 +1191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1158,6 +1201,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1471,7 +1516,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V114"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1616,7 +1661,7 @@
       <c r="A5" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="8" t="s">
         <v>273</v>
       </c>
       <c r="C5" s="4" t="s">
@@ -1634,7 +1679,7 @@
       <c r="G5" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="8" t="s">
         <v>273</v>
       </c>
       <c r="I5" s="4" t="s">
@@ -1672,7 +1717,7 @@
       <c r="A6" s="5" t="s">
         <v>245</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="8" t="s">
         <v>274</v>
       </c>
       <c r="C6" s="5" t="s">
@@ -1690,7 +1735,7 @@
       <c r="G6" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="8" t="s">
         <v>274</v>
       </c>
       <c r="I6" s="5" t="s">
@@ -1820,7 +1865,7 @@
       <c r="M8" s="5" t="s">
         <v>290</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="N8" s="8" t="s">
         <v>273</v>
       </c>
       <c r="O8" s="5" t="s">
@@ -1876,7 +1921,7 @@
       <c r="M9" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="N9" s="8" t="s">
         <v>274</v>
       </c>
       <c r="O9" s="5" t="s">
@@ -2456,7 +2501,7 @@
       <c r="A20" s="5" t="s">
         <v>259</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="8" t="s">
         <v>275</v>
       </c>
       <c r="C20" s="5" t="s">
@@ -2530,7 +2575,7 @@
       <c r="G21" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="H21" s="5" t="s">
+      <c r="H21" s="8" t="s">
         <v>276</v>
       </c>
       <c r="I21" s="5" t="s">
@@ -2642,7 +2687,7 @@
       <c r="G23" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="H23" s="5" t="s">
+      <c r="H23" s="8" t="s">
         <v>277</v>
       </c>
       <c r="I23" s="5" t="s">
@@ -2789,7 +2834,7 @@
       <c r="A26" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="8" t="s">
         <v>276</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -3089,7 +3134,7 @@
       <c r="A32" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="8" t="s">
         <v>277</v>
       </c>
       <c r="C32" s="5" t="s">
@@ -3312,7 +3357,7 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="8" t="s">
         <v>278</v>
       </c>
       <c r="C37" s="5" t="s">
@@ -4107,7 +4152,7 @@
       <c r="M67" s="5" t="s">
         <v>260</v>
       </c>
-      <c r="N67" s="5" t="s">
+      <c r="N67" s="8" t="s">
         <v>275</v>
       </c>
       <c r="O67" s="5" t="s">
@@ -4227,7 +4272,7 @@
       <c r="M73" s="5" t="s">
         <v>346</v>
       </c>
-      <c r="N73" s="5" t="s">
+      <c r="N73" s="8" t="s">
         <v>276</v>
       </c>
       <c r="O73" s="5" t="s">
@@ -4381,7 +4426,7 @@
       </c>
     </row>
     <row r="81" spans="14:18" x14ac:dyDescent="0.25">
-      <c r="N81" s="5" t="s">
+      <c r="N81" s="8" t="s">
         <v>277</v>
       </c>
       <c r="O81" s="5" t="s">
@@ -4716,6 +4761,94 @@
       </c>
       <c r="R114" t="s">
         <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE29EB32-4035-4508-8E7F-C33AD81BA39D}">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>350</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>353</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>351</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>